<commit_message>
11 enero 2022 v1
</commit_message>
<xml_diff>
--- a/_downloads/f52a95a041023a4c83e993531fb46e55/Indicadores liquidez-endeuda-renta-H&M.xlsx
+++ b/_downloads/f52a95a041023a4c83e993531fb46e55/Indicadores liquidez-endeuda-renta-H&M.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\UNAL\ADMINISTRACIÓN FINANCIERA\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{178CFB9A-66B4-43D0-9ACE-B78C556CBB8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBE5A964-61B5-419F-AD5C-B040DDF218B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{88032940-B68D-4784-94D6-624C0E8A8768}"/>
   </bookViews>
@@ -21326,2175 +21326,6 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>657225</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>200025</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>229783</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>24897</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="15" name="CuadroTexto 24">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000F000000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="14792325" y="7115175"/>
-              <a:ext cx="1858558" cy="453522"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr wrap="square">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle>
-              <a:defPPr>
-                <a:defRPr lang="es-CO"/>
-              </a:defPPr>
-              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl1pPr>
-              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl2pPr>
-              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl3pPr>
-              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl4pPr>
-              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl5pPr>
-              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl6pPr>
-              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl7pPr>
-              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl8pPr>
-              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl9pPr>
-            </a:lstStyle>
-            <a:p>
-              <a:pPr/>
-              <a14:m>
-                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                    <m:r>
-                      <m:rPr>
-                        <m:nor/>
-                      </m:rPr>
-                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                      </a:rPr>
-                      <m:t>ROA</m:t>
-                    </m:r>
-                    <m:r>
-                      <m:rPr>
-                        <m:nor/>
-                      </m:rPr>
-                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                      </a:rPr>
-                      <m:t> = </m:t>
-                    </m:r>
-                    <m:f>
-                      <m:fPr>
-                        <m:ctrlPr>
-                          <a:rPr lang="es-CO" sz="1200" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:fPr>
-                      <m:num>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Utilidad</m:t>
-                        </m:r>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t> </m:t>
-                        </m:r>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Neta</m:t>
-                        </m:r>
-                      </m:num>
-                      <m:den>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Activos</m:t>
-                        </m:r>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t> </m:t>
-                        </m:r>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Totales</m:t>
-                        </m:r>
-                      </m:den>
-                    </m:f>
-                  </m:oMath>
-                </m:oMathPara>
-              </a14:m>
-              <a:endParaRPr lang="es-CO" sz="1200"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Choice>
-      <mc:Fallback xmlns="">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="15" name="CuadroTexto 24">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000F000000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="14792325" y="7115175"/>
-              <a:ext cx="1858558" cy="453522"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr wrap="square">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle>
-              <a:defPPr>
-                <a:defRPr lang="es-CO"/>
-              </a:defPPr>
-              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl1pPr>
-              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl2pPr>
-              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl3pPr>
-              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl4pPr>
-              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl5pPr>
-              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl6pPr>
-              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl7pPr>
-              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl8pPr>
-              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl9pPr>
-            </a:lstStyle>
-            <a:p>
-              <a:pPr/>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>"ROA = </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-CO" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>" </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t> "Utilidad Neta</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>" </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-CO" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>/</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>"</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>Activos Totales</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>" </a:t>
-              </a:r>
-              <a:endParaRPr lang="es-CO" sz="1200"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>619125</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>190500</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>266403</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>10371</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="16" name="CuadroTexto 26">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000010000000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="14754225" y="7734300"/>
-              <a:ext cx="2695278" cy="448521"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr wrap="square">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle>
-              <a:defPPr>
-                <a:defRPr lang="es-CO"/>
-              </a:defPPr>
-              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl1pPr>
-              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl2pPr>
-              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl3pPr>
-              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl4pPr>
-              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl5pPr>
-              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl6pPr>
-              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl7pPr>
-              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl8pPr>
-              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl9pPr>
-            </a:lstStyle>
-            <a:p>
-              <a:pPr/>
-              <a14:m>
-                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                    <m:r>
-                      <m:rPr>
-                        <m:nor/>
-                      </m:rPr>
-                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                      </a:rPr>
-                      <m:t>ROA</m:t>
-                    </m:r>
-                    <m:r>
-                      <m:rPr>
-                        <m:nor/>
-                      </m:rPr>
-                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                      </a:rPr>
-                      <m:t> </m:t>
-                    </m:r>
-                    <m:r>
-                      <m:rPr>
-                        <m:nor/>
-                      </m:rPr>
-                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                      </a:rPr>
-                      <m:t>Operacional</m:t>
-                    </m:r>
-                    <m:r>
-                      <m:rPr>
-                        <m:nor/>
-                      </m:rPr>
-                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                      </a:rPr>
-                      <m:t> = </m:t>
-                    </m:r>
-                    <m:f>
-                      <m:fPr>
-                        <m:ctrlPr>
-                          <a:rPr lang="es-CO" sz="1200" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:fPr>
-                      <m:num>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>EBIT</m:t>
-                        </m:r>
-                      </m:num>
-                      <m:den>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Activos</m:t>
-                        </m:r>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t> </m:t>
-                        </m:r>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Totales</m:t>
-                        </m:r>
-                      </m:den>
-                    </m:f>
-                  </m:oMath>
-                </m:oMathPara>
-              </a14:m>
-              <a:endParaRPr lang="es-CO" sz="1200"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Choice>
-      <mc:Fallback xmlns="">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="16" name="CuadroTexto 26">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000010000000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="14754225" y="7734300"/>
-              <a:ext cx="2695278" cy="448521"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr wrap="square">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle>
-              <a:defPPr>
-                <a:defRPr lang="es-CO"/>
-              </a:defPPr>
-              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl1pPr>
-              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl2pPr>
-              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl3pPr>
-              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl4pPr>
-              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl5pPr>
-              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl6pPr>
-              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl7pPr>
-              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl8pPr>
-              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl9pPr>
-            </a:lstStyle>
-            <a:p>
-              <a:pPr/>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>"ROA Operacional = </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-CO" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>" </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" i="0">
-                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t> "EBIT</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>" </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-CO" sz="1200" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>/</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>"</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" i="0">
-                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>Activos Totales</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>" </a:t>
-              </a:r>
-              <a:endParaRPr lang="es-CO" sz="1200"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>609600</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>66675</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>744133</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>101097</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="17" name="CuadroTexto 25">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000011000000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="14744700" y="8239125"/>
-              <a:ext cx="1658533" cy="453522"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr wrap="square">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle>
-              <a:defPPr>
-                <a:defRPr lang="es-CO"/>
-              </a:defPPr>
-              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl1pPr>
-              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl2pPr>
-              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl3pPr>
-              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl4pPr>
-              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl5pPr>
-              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl6pPr>
-              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl7pPr>
-              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl8pPr>
-              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl9pPr>
-            </a:lstStyle>
-            <a:p>
-              <a:pPr/>
-              <a14:m>
-                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                    <m:r>
-                      <m:rPr>
-                        <m:nor/>
-                      </m:rPr>
-                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                      </a:rPr>
-                      <m:t>ROE</m:t>
-                    </m:r>
-                    <m:r>
-                      <m:rPr>
-                        <m:nor/>
-                      </m:rPr>
-                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                      </a:rPr>
-                      <m:t> =</m:t>
-                    </m:r>
-                    <m:f>
-                      <m:fPr>
-                        <m:ctrlPr>
-                          <a:rPr lang="es-CO" sz="1200" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:fPr>
-                      <m:num>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Utilidad</m:t>
-                        </m:r>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t> </m:t>
-                        </m:r>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Neta</m:t>
-                        </m:r>
-                      </m:num>
-                      <m:den>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Patrimonio</m:t>
-                        </m:r>
-                      </m:den>
-                    </m:f>
-                  </m:oMath>
-                </m:oMathPara>
-              </a14:m>
-              <a:endParaRPr lang="es-CO" sz="1200"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Choice>
-      <mc:Fallback xmlns="">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="17" name="CuadroTexto 25">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000011000000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="14744700" y="8239125"/>
-              <a:ext cx="1658533" cy="453522"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr wrap="square">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle>
-              <a:defPPr>
-                <a:defRPr lang="es-CO"/>
-              </a:defPPr>
-              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl1pPr>
-              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl2pPr>
-              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl3pPr>
-              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl4pPr>
-              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl5pPr>
-              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl6pPr>
-              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl7pPr>
-              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl8pPr>
-              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl9pPr>
-            </a:lstStyle>
-            <a:p>
-              <a:pPr/>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>"ROE =</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-CO" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>" </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" i="0">
-                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t> "Utilidad Neta</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>" </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-CO" sz="1200" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>/</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>"</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" i="0">
-                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>Patrimonio</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>" </a:t>
-              </a:r>
-              <a:endParaRPr lang="es-CO" sz="1200"/>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>466724</xdr:colOff>
-      <xdr:row>42</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>544977</xdr:colOff>
-      <xdr:row>43</xdr:row>
-      <xdr:rowOff>189739</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="18" name="CuadroTexto 19">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000012000000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="14601824" y="8839200"/>
-              <a:ext cx="5412253" cy="361189"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle>
-              <a:defPPr>
-                <a:defRPr lang="es-CO"/>
-              </a:defPPr>
-              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl1pPr>
-              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl2pPr>
-              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl3pPr>
-              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl4pPr>
-              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl5pPr>
-              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl6pPr>
-              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl7pPr>
-              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl8pPr>
-              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl9pPr>
-            </a:lstStyle>
-            <a:p>
-              <a:pPr/>
-              <a14:m>
-                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                  <m:oMathParaPr>
-                    <m:jc m:val="centerGroup"/>
-                  </m:oMathParaPr>
-                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
-                    <m:r>
-                      <m:rPr>
-                        <m:nor/>
-                      </m:rPr>
-                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                      </a:rPr>
-                      <m:t>ROE</m:t>
-                    </m:r>
-                    <m:r>
-                      <m:rPr>
-                        <m:nor/>
-                      </m:rPr>
-                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                      </a:rPr>
-                      <m:t> = </m:t>
-                    </m:r>
-                    <m:f>
-                      <m:fPr>
-                        <m:ctrlPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:fPr>
-                      <m:num>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                            <a:solidFill>
-                              <a:srgbClr val="14085C"/>
-                            </a:solidFill>
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Utilidad</m:t>
-                        </m:r>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                            <a:solidFill>
-                              <a:srgbClr val="14085C"/>
-                            </a:solidFill>
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t> </m:t>
-                        </m:r>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                            <a:solidFill>
-                              <a:srgbClr val="14085C"/>
-                            </a:solidFill>
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Neta</m:t>
-                        </m:r>
-                      </m:num>
-                      <m:den>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Ventas</m:t>
-                        </m:r>
-                      </m:den>
-                    </m:f>
-                    <m:r>
-                      <m:rPr>
-                        <m:nor/>
-                      </m:rPr>
-                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t> </m:t>
-                    </m:r>
-                    <m:r>
-                      <m:rPr>
-                        <m:nor/>
-                      </m:rPr>
-                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                      </a:rPr>
-                      <m:t>× </m:t>
-                    </m:r>
-                    <m:f>
-                      <m:fPr>
-                        <m:ctrlPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                            <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:fPr>
-                      <m:num>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Ventas</m:t>
-                        </m:r>
-                      </m:num>
-                      <m:den>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Activos</m:t>
-                        </m:r>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t> </m:t>
-                        </m:r>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Totales</m:t>
-                        </m:r>
-                      </m:den>
-                    </m:f>
-                    <m:r>
-                      <m:rPr>
-                        <m:nor/>
-                      </m:rPr>
-                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                        <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                      </a:rPr>
-                      <m:t> </m:t>
-                    </m:r>
-                    <m:r>
-                      <m:rPr>
-                        <m:nor/>
-                      </m:rPr>
-                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                      </a:rPr>
-                      <m:t>×</m:t>
-                    </m:r>
-                    <m:f>
-                      <m:fPr>
-                        <m:ctrlPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                            <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:fPr>
-                      <m:num>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Activos</m:t>
-                        </m:r>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t> </m:t>
-                        </m:r>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Totales</m:t>
-                        </m:r>
-                      </m:num>
-                      <m:den>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                            <a:solidFill>
-                              <a:srgbClr val="14085C"/>
-                            </a:solidFill>
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Patrimonio</m:t>
-                        </m:r>
-                      </m:den>
-                    </m:f>
-                    <m:r>
-                      <m:rPr>
-                        <m:nor/>
-                      </m:rPr>
-                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                      </a:rPr>
-                      <m:t>=</m:t>
-                    </m:r>
-                    <m:f>
-                      <m:fPr>
-                        <m:ctrlPr>
-                          <a:rPr lang="es-MX" sz="1200" i="1">
-                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          </a:rPr>
-                        </m:ctrlPr>
-                      </m:fPr>
-                      <m:num>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" i="0">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Utilidad</m:t>
-                        </m:r>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" i="0">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t> </m:t>
-                        </m:r>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" i="0">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Neta</m:t>
-                        </m:r>
-                      </m:num>
-                      <m:den>
-                        <m:r>
-                          <m:rPr>
-                            <m:nor/>
-                          </m:rPr>
-                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                          </a:rPr>
-                          <m:t>Patrimonio</m:t>
-                        </m:r>
-                      </m:den>
-                    </m:f>
-                  </m:oMath>
-                </m:oMathPara>
-              </a14:m>
-              <a:endParaRPr lang="es-CO" sz="1200">
-                <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              </a:endParaRPr>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Choice>
-      <mc:Fallback xmlns="">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="18" name="CuadroTexto 19">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000012000000}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvSpPr txBox="1"/>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="14601824" y="8839200"/>
-              <a:ext cx="5412253" cy="361189"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:noFill/>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0">
-              <a:spAutoFit/>
-            </a:bodyPr>
-            <a:lstStyle>
-              <a:defPPr>
-                <a:defRPr lang="es-CO"/>
-              </a:defPPr>
-              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl1pPr>
-              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl2pPr>
-              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl3pPr>
-              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl4pPr>
-              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl5pPr>
-              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl6pPr>
-              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl7pPr>
-              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl8pPr>
-              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
-                <a:defRPr sz="1800" kern="1200">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1"/>
-                  </a:solidFill>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
-                </a:defRPr>
-              </a:lvl9pPr>
-            </a:lstStyle>
-            <a:p>
-              <a:pPr/>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>"ROE = " </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:solidFill>
-                    <a:srgbClr val="14085C"/>
-                  </a:solidFill>
-                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t> "Utilidad Neta</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:solidFill>
-                    <a:srgbClr val="14085C"/>
-                  </a:solidFill>
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>" /"</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>Ventas</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>"  "</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t> </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>× </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>" </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t> "Ventas</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>" </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>/"</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>Activos Totales</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>" </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t> "</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                </a:rPr>
-                <a:t> </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>×</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>" </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t> "Activos Totales</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>" </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>/</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:solidFill>
-                    <a:srgbClr val="14085C"/>
-                  </a:solidFill>
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>"</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:solidFill>
-                    <a:srgbClr val="14085C"/>
-                  </a:solidFill>
-                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>Patrimonio</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:solidFill>
-                    <a:srgbClr val="14085C"/>
-                  </a:solidFill>
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>"  "</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>=" </a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" i="0">
-                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t> "Utilidad Neta</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>" /</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>"</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>Patrimonio</a:t>
-              </a:r>
-              <a:r>
-                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
-                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                </a:rPr>
-                <a:t>" </a:t>
-              </a:r>
-              <a:endParaRPr lang="es-CO" sz="1200">
-                <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-                <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
-              </a:endParaRPr>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
       <xdr:col>10</xdr:col>
       <xdr:colOff>952500</xdr:colOff>
       <xdr:row>45</xdr:row>
@@ -23506,8 +21337,8 @@
       <xdr:row>46</xdr:row>
       <xdr:rowOff>45253</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="19" name="CuadroTexto 18">
@@ -23799,7 +21630,7 @@
                         <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
                         <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
                       </a:rPr>
-                      <m:t>Apalancamiento</m:t>
+                      <m:t>Multiplicador</m:t>
                     </m:r>
                     <m:r>
                       <m:rPr>
@@ -23821,7 +21652,29 @@
                         <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
                         <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
                       </a:rPr>
-                      <m:t>financiero</m:t>
+                      <m:t>de</m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                      </a:rPr>
+                      <m:t>Capital</m:t>
                     </m:r>
                   </m:oMath>
                 </m:oMathPara>
@@ -23835,7 +21688,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback xmlns="">
+      <mc:Fallback>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="19" name="CuadroTexto 18">
@@ -23964,7 +21817,7 @@
                   <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
                   <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
                 </a:rPr>
-                <a:t>"ROE = Margen Neto × Rotación de Activos × Apalancamiento financiero</a:t>
+                <a:t>"ROE = Margen Neto × Rotación de Activos × Multiplicador de Capital</a:t>
               </a:r>
               <a:r>
                 <a:rPr lang="es-CO" sz="1200" b="0" i="0">
@@ -24774,7 +22627,7 @@
       <xdr:col>16</xdr:col>
       <xdr:colOff>466725</xdr:colOff>
       <xdr:row>22</xdr:row>
-      <xdr:rowOff>82242</xdr:rowOff>
+      <xdr:rowOff>88627</xdr:rowOff>
     </xdr:to>
     <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
       <mc:Choice Requires="a14">
@@ -24791,8 +22644,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="14792325" y="4343400"/>
-              <a:ext cx="3619500" cy="348942"/>
+              <a:off x="14856802" y="4402015"/>
+              <a:ext cx="3619500" cy="361189"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -24968,9 +22821,9 @@
                               <a:schemeClr val="tx1"/>
                             </a:solidFill>
                             <a:effectLst/>
-                            <a:latin typeface="+mn-lt"/>
-                            <a:ea typeface="+mn-ea"/>
-                            <a:cs typeface="+mn-cs"/>
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
                           </a:rPr>
                           <m:t>Promedio</m:t>
                         </m:r>
@@ -24983,9 +22836,9 @@
                               <a:schemeClr val="tx1"/>
                             </a:solidFill>
                             <a:effectLst/>
-                            <a:latin typeface="+mn-lt"/>
-                            <a:ea typeface="+mn-ea"/>
-                            <a:cs typeface="+mn-cs"/>
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
                           </a:rPr>
                           <m:t> </m:t>
                         </m:r>
@@ -24998,9 +22851,9 @@
                               <a:schemeClr val="tx1"/>
                             </a:solidFill>
                             <a:effectLst/>
-                            <a:latin typeface="+mn-lt"/>
-                            <a:ea typeface="+mn-ea"/>
-                            <a:cs typeface="+mn-cs"/>
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
                           </a:rPr>
                           <m:t>Pasivo</m:t>
                         </m:r>
@@ -25013,9 +22866,9 @@
                               <a:schemeClr val="tx1"/>
                             </a:solidFill>
                             <a:effectLst/>
-                            <a:latin typeface="+mn-lt"/>
-                            <a:ea typeface="+mn-ea"/>
-                            <a:cs typeface="+mn-cs"/>
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
                           </a:rPr>
                           <m:t> </m:t>
                         </m:r>
@@ -25028,9 +22881,9 @@
                               <a:schemeClr val="tx1"/>
                             </a:solidFill>
                             <a:effectLst/>
-                            <a:latin typeface="+mn-lt"/>
-                            <a:ea typeface="+mn-ea"/>
-                            <a:cs typeface="+mn-cs"/>
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
                           </a:rPr>
                           <m:t>Total</m:t>
                         </m:r>
@@ -25097,8 +22950,8 @@
           </xdr:nvSpPr>
           <xdr:spPr>
             <a:xfrm>
-              <a:off x="14792325" y="4343400"/>
-              <a:ext cx="3619500" cy="348942"/>
+              <a:off x="14856802" y="4402015"/>
+              <a:ext cx="3619500" cy="361189"/>
             </a:xfrm>
             <a:prstGeom prst="rect">
               <a:avLst/>
@@ -25220,9 +23073,9 @@
                     <a:schemeClr val="tx1"/>
                   </a:solidFill>
                   <a:effectLst/>
-                  <a:latin typeface="+mn-lt"/>
-                  <a:ea typeface="+mn-ea"/>
-                  <a:cs typeface="+mn-cs"/>
+                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
                 </a:rPr>
                 <a:t> "Promedio Pasivo Total</a:t>
               </a:r>
@@ -25885,6 +23738,2370 @@
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>644769</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>128953</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>654293</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>157514</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="32" name="CuadroTexto 24">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5024BF4C-304A-4A76-B91C-C9243851FE5F}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="14844346" y="7778261"/>
+              <a:ext cx="2295524" cy="453522"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr wrap="square">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle>
+              <a:defPPr>
+                <a:defRPr lang="es-CO"/>
+              </a:defPPr>
+              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl1pPr>
+              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl2pPr>
+              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl3pPr>
+              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl4pPr>
+              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl5pPr>
+              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl6pPr>
+              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl7pPr>
+              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl8pPr>
+              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl9pPr>
+            </a:lstStyle>
+            <a:p>
+              <a:pPr/>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMathParaPr>
+                    <m:jc m:val="centerGroup"/>
+                  </m:oMathParaPr>
+                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                      </a:rPr>
+                      <m:t>ROA</m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                      </a:rPr>
+                      <m:t> = </m:t>
+                    </m:r>
+                    <m:f>
+                      <m:fPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="es-CO" sz="1200" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:fPr>
+                      <m:num>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Utilidad</m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t> </m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Neta</m:t>
+                        </m:r>
+                      </m:num>
+                      <m:den>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Prom</m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>. </m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Activos</m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t> </m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Totales</m:t>
+                        </m:r>
+                      </m:den>
+                    </m:f>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="es-CO" sz="1200"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Choice>
+      <mc:Fallback xmlns="">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="32" name="CuadroTexto 24">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5024BF4C-304A-4A76-B91C-C9243851FE5F}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="14844346" y="7778261"/>
+              <a:ext cx="2295524" cy="453522"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr wrap="square">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle>
+              <a:defPPr>
+                <a:defRPr lang="es-CO"/>
+              </a:defPPr>
+              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl1pPr>
+              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl2pPr>
+              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl3pPr>
+              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl4pPr>
+              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl5pPr>
+              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl6pPr>
+              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl7pPr>
+              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl8pPr>
+              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl9pPr>
+            </a:lstStyle>
+            <a:p>
+              <a:pPr/>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>"ROA = </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-CO" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>" </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t> "Utilidad Neta</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>" </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-CO" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>/</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>"</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>Prom. Activos Totales</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>" </a:t>
+              </a:r>
+              <a:endParaRPr lang="es-CO" sz="1200"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>597875</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>183173</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>740020</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>206732</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="39" name="CuadroTexto 26">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{966EB4B3-8014-4B39-BEC1-0F675D5840B2}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="14797452" y="7195038"/>
+              <a:ext cx="3190145" cy="448521"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr wrap="square">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle>
+              <a:defPPr>
+                <a:defRPr lang="es-CO"/>
+              </a:defPPr>
+              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl1pPr>
+              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl2pPr>
+              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl3pPr>
+              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl4pPr>
+              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl5pPr>
+              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl6pPr>
+              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl7pPr>
+              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl8pPr>
+              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl9pPr>
+            </a:lstStyle>
+            <a:p>
+              <a:pPr/>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMathParaPr>
+                    <m:jc m:val="centerGroup"/>
+                  </m:oMathParaPr>
+                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                      </a:rPr>
+                      <m:t>ROA</m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                      </a:rPr>
+                      <m:t>Operacional</m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                      </a:rPr>
+                      <m:t> = </m:t>
+                    </m:r>
+                    <m:f>
+                      <m:fPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="es-CO" sz="1200" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:fPr>
+                      <m:num>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>EBIT</m:t>
+                        </m:r>
+                      </m:num>
+                      <m:den>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Prom</m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>. </m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Activos</m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t> </m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Totales</m:t>
+                        </m:r>
+                      </m:den>
+                    </m:f>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="es-CO" sz="1200"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Choice>
+      <mc:Fallback xmlns="">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="39" name="CuadroTexto 26">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{966EB4B3-8014-4B39-BEC1-0F675D5840B2}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="14797452" y="7195038"/>
+              <a:ext cx="3190145" cy="448521"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr wrap="square">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle>
+              <a:defPPr>
+                <a:defRPr lang="es-CO"/>
+              </a:defPPr>
+              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl1pPr>
+              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl2pPr>
+              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl3pPr>
+              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl4pPr>
+              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl5pPr>
+              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl6pPr>
+              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl7pPr>
+              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl8pPr>
+              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl9pPr>
+            </a:lstStyle>
+            <a:p>
+              <a:pPr/>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>"ROA Operacional = </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-CO" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>" </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" i="0">
+                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t> "EBIT</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>" </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-CO" sz="1200" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>/</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>"</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>Prom. A</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" i="0">
+                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>ctivos Totales</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>" </a:t>
+              </a:r>
+              <a:endParaRPr lang="es-CO" sz="1200"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>530467</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>95249</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>380999</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>123809</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="42" name="CuadroTexto 25">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AB17B0B2-D4BD-4795-8031-A745C077EE99}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="14730044" y="8381999"/>
+              <a:ext cx="2136532" cy="453522"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr wrap="square">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle>
+              <a:defPPr>
+                <a:defRPr lang="es-CO"/>
+              </a:defPPr>
+              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl1pPr>
+              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl2pPr>
+              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl3pPr>
+              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl4pPr>
+              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl5pPr>
+              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl6pPr>
+              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl7pPr>
+              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl8pPr>
+              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl9pPr>
+            </a:lstStyle>
+            <a:p>
+              <a:pPr/>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMathParaPr>
+                    <m:jc m:val="centerGroup"/>
+                  </m:oMathParaPr>
+                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                      </a:rPr>
+                      <m:t>ROE</m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                      </a:rPr>
+                      <m:t> =</m:t>
+                    </m:r>
+                    <m:f>
+                      <m:fPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="es-CO" sz="1200" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:fPr>
+                      <m:num>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Utilidad</m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t> </m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Neta</m:t>
+                        </m:r>
+                      </m:num>
+                      <m:den>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>P</m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>rom</m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>. </m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Patrimonio</m:t>
+                        </m:r>
+                      </m:den>
+                    </m:f>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="es-CO" sz="1200"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Choice>
+      <mc:Fallback xmlns="">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="42" name="CuadroTexto 25">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AB17B0B2-D4BD-4795-8031-A745C077EE99}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="14730044" y="8381999"/>
+              <a:ext cx="2136532" cy="453522"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr wrap="square">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle>
+              <a:defPPr>
+                <a:defRPr lang="es-CO"/>
+              </a:defPPr>
+              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl1pPr>
+              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl2pPr>
+              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl3pPr>
+              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl4pPr>
+              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl5pPr>
+              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl6pPr>
+              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl7pPr>
+              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl8pPr>
+              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl9pPr>
+            </a:lstStyle>
+            <a:p>
+              <a:pPr/>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>"ROE =</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-CO" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>" </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" i="0">
+                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t> "Utilidad Neta</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>" </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-CO" sz="1200" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>/</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>"</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" i="0">
+                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>P</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>rom. P</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" i="0">
+                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>atrimonio</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>" </a:t>
+              </a:r>
+              <a:endParaRPr lang="es-CO" sz="1200"/>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>754671</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>125290</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>117231</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>61517</xdr:rowOff>
+    </xdr:to>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="43" name="CuadroTexto 19">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{57CF5900-5E1B-4EFF-A592-1D359F66573F}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="14954248" y="9049482"/>
+              <a:ext cx="6220560" cy="361189"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle>
+              <a:defPPr>
+                <a:defRPr lang="es-CO"/>
+              </a:defPPr>
+              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl1pPr>
+              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl2pPr>
+              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl3pPr>
+              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl4pPr>
+              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl5pPr>
+              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl6pPr>
+              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl7pPr>
+              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl8pPr>
+              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl9pPr>
+            </a:lstStyle>
+            <a:p>
+              <a:pPr/>
+              <a14:m>
+                <m:oMathPara xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                  <m:oMathParaPr>
+                    <m:jc m:val="centerGroup"/>
+                  </m:oMathParaPr>
+                  <m:oMath xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math">
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                      </a:rPr>
+                      <m:t>ROE</m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                      </a:rPr>
+                      <m:t> = </m:t>
+                    </m:r>
+                    <m:f>
+                      <m:fPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:fPr>
+                      <m:num>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:solidFill>
+                              <a:srgbClr val="14085C"/>
+                            </a:solidFill>
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Utilidad</m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:solidFill>
+                              <a:srgbClr val="14085C"/>
+                            </a:solidFill>
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t> </m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:solidFill>
+                              <a:srgbClr val="14085C"/>
+                            </a:solidFill>
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Neta</m:t>
+                        </m:r>
+                      </m:num>
+                      <m:den>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Ventas</m:t>
+                        </m:r>
+                      </m:den>
+                    </m:f>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                      </a:rPr>
+                      <m:t>× </m:t>
+                    </m:r>
+                    <m:f>
+                      <m:fPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:fPr>
+                      <m:num>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Ventas</m:t>
+                        </m:r>
+                      </m:num>
+                      <m:den>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Prom</m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>. </m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Activos</m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t> </m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Totales</m:t>
+                        </m:r>
+                      </m:den>
+                    </m:f>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                        <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                        <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                      </a:rPr>
+                      <m:t> </m:t>
+                    </m:r>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                      </a:rPr>
+                      <m:t>×</m:t>
+                    </m:r>
+                    <m:f>
+                      <m:fPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                            <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:fPr>
+                      <m:num>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Prom</m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>. </m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Activos</m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t> </m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Totales</m:t>
+                        </m:r>
+                      </m:num>
+                      <m:den>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:solidFill>
+                              <a:srgbClr val="14085C"/>
+                            </a:solidFill>
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Prom</m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:solidFill>
+                              <a:srgbClr val="14085C"/>
+                            </a:solidFill>
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>. </m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:solidFill>
+                              <a:srgbClr val="14085C"/>
+                            </a:solidFill>
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Patrimonio</m:t>
+                        </m:r>
+                      </m:den>
+                    </m:f>
+                    <m:r>
+                      <m:rPr>
+                        <m:nor/>
+                      </m:rPr>
+                      <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                        <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                        <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                      </a:rPr>
+                      <m:t>=</m:t>
+                    </m:r>
+                    <m:f>
+                      <m:fPr>
+                        <m:ctrlPr>
+                          <a:rPr lang="es-MX" sz="1200" i="1">
+                            <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                          </a:rPr>
+                        </m:ctrlPr>
+                      </m:fPr>
+                      <m:num>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Utilidad</m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t> </m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Neta</m:t>
+                        </m:r>
+                      </m:num>
+                      <m:den>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Prom</m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>. </m:t>
+                        </m:r>
+                        <m:r>
+                          <m:rPr>
+                            <m:nor/>
+                          </m:rPr>
+                          <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                            <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                            <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                          </a:rPr>
+                          <m:t>Patrimonio</m:t>
+                        </m:r>
+                      </m:den>
+                    </m:f>
+                  </m:oMath>
+                </m:oMathPara>
+              </a14:m>
+              <a:endParaRPr lang="es-CO" sz="1200">
+                <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+              </a:endParaRPr>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Choice>
+      <mc:Fallback xmlns="">
+        <xdr:sp macro="" textlink="">
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="43" name="CuadroTexto 19">
+              <a:extLst>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{57CF5900-5E1B-4EFF-A592-1D359F66573F}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr txBox="1"/>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="14954248" y="9049482"/>
+              <a:ext cx="6220560" cy="361189"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect">
+              <a:avLst/>
+            </a:prstGeom>
+            <a:noFill/>
+          </xdr:spPr>
+          <xdr:txBody>
+            <a:bodyPr wrap="square" lIns="0" tIns="0" rIns="0" bIns="0" rtlCol="0">
+              <a:spAutoFit/>
+            </a:bodyPr>
+            <a:lstStyle>
+              <a:defPPr>
+                <a:defRPr lang="es-CO"/>
+              </a:defPPr>
+              <a:lvl1pPr marL="0" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl1pPr>
+              <a:lvl2pPr marL="457200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl2pPr>
+              <a:lvl3pPr marL="914400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl3pPr>
+              <a:lvl4pPr marL="1371600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl4pPr>
+              <a:lvl5pPr marL="1828800" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl5pPr>
+              <a:lvl6pPr marL="2286000" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl6pPr>
+              <a:lvl7pPr marL="2743200" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl7pPr>
+              <a:lvl8pPr marL="3200400" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl8pPr>
+              <a:lvl9pPr marL="3657600" algn="l" defTabSz="914400" rtl="0" eaLnBrk="1" latinLnBrk="0" hangingPunct="1">
+                <a:defRPr sz="1800" kern="1200">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:lvl9pPr>
+            </a:lstStyle>
+            <a:p>
+              <a:pPr/>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>"ROE = " </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:solidFill>
+                    <a:srgbClr val="14085C"/>
+                  </a:solidFill>
+                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t> "Utilidad Neta</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:solidFill>
+                    <a:srgbClr val="14085C"/>
+                  </a:solidFill>
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>" /"</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>Ventas</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>"  "</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t> </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>× </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>" </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t> "Ventas</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>" </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>/"</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>Prom. Activos Totales</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>" </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t> "</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                </a:rPr>
+                <a:t> </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>×</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>" </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t> "Prom. Activos Totales</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>" </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>/</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:solidFill>
+                    <a:srgbClr val="14085C"/>
+                  </a:solidFill>
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>"</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:solidFill>
+                    <a:srgbClr val="14085C"/>
+                  </a:solidFill>
+                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>Prom. Patrimonio</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:solidFill>
+                    <a:srgbClr val="14085C"/>
+                  </a:solidFill>
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>"  "</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>=" </a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" i="0">
+                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t> "Utilidad Neta</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>" /</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>"</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>Prom. Patrimonio</a:t>
+              </a:r>
+              <a:r>
+                <a:rPr lang="es-MX" sz="1200" b="0" i="0">
+                  <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
+                  <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                  <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                </a:rPr>
+                <a:t>" </a:t>
+              </a:r>
+              <a:endParaRPr lang="es-CO" sz="1200">
+                <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+                <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
+              </a:endParaRPr>
+            </a:p>
+          </xdr:txBody>
+        </xdr:sp>
+      </mc:Fallback>
+    </mc:AlternateContent>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>

</xml_diff>